<commit_message>
avniproject/avni-webapp#1780 | Refine dataset
</commit_message>
<xml_diff>
--- a/requirements/rules_ai_automation.xlsx
+++ b/requirements/rules_ai_automation.xlsx
@@ -23677,7 +23677,7 @@
     <outlinePr summaryBelow="0" summaryRight="0"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D25"/>
+  <dimension ref="A1:D23"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="12.63" defaultRowHeight="15" customHeight="1"/>
   <cols>
     <col width="22" customWidth="1" style="11" min="1" max="1"/>
@@ -23767,7 +23767,7 @@
       </c>
       <c r="D3" s="13" t="inlineStr">
         <is>
-          <t>block cancelling an encounter on or after its scheduled date</t>
+          <t>block cancelling an encounter before its scheduled date</t>
         </is>
       </c>
     </row>
@@ -23800,7 +23800,7 @@
       </c>
       <c r="D4" s="13" t="inlineStr">
         <is>
-          <t>block cancelling an encounter within N days of its scheduled date, or after the program has been exited</t>
+          <t>block cancelling an encounter more than N days before its scheduled date (skip the check once the program is exited)</t>
         </is>
       </c>
     </row>
@@ -23843,7 +23843,7 @@
       </c>
       <c r="D5" s="13" t="inlineStr">
         <is>
-          <t>block saving when the visit is overdue (past maxVisitDateTime) or being filled in a month before the schedule month</t>
+          <t>block saving when the visit is overdue or its date is before the scheduled date</t>
         </is>
       </c>
     </row>
@@ -23879,7 +23879,7 @@
       </c>
       <c r="D6" s="13" t="inlineStr">
         <is>
-          <t>block saving when the encounter is filled too far before its scheduled date, with the allowed gap varying by visit type</t>
+          <t>block saving when the encounter is filled more than N weeks before its scheduled date</t>
         </is>
       </c>
     </row>
@@ -23928,7 +23928,7 @@
       </c>
       <c r="D7" s="13" t="inlineStr">
         <is>
-          <t>lock the encounter/registration date after the first save so it can't be changed on subsequent edits</t>
+          <t>lock the entry date after the first save so it can't be changed on subsequent edits</t>
         </is>
       </c>
     </row>
@@ -23992,7 +23992,7 @@
       </c>
       <c r="D8" s="13" t="inlineStr">
         <is>
-          <t>lock the encounter date across edits and require at least one image or file in the grouped upload section</t>
+          <t>lock the encounter date across edits and require at least one supporting media or file in the form</t>
         </is>
       </c>
     </row>
@@ -24022,7 +24022,7 @@
       </c>
       <c r="D9" s="13" t="inlineStr">
         <is>
-          <t>block saving when the sum of category counts exceeds the parent total (e.g. positive cases &lt;= total screened)</t>
+          <t>block saving when one observation count exceeds another logically-larger one (e.g. beneficiaries received &gt; beneficiaries requested)</t>
         </is>
       </c>
     </row>
@@ -24060,7 +24060,7 @@
       </c>
       <c r="D10" s="13" t="inlineStr">
         <is>
-          <t>block saving when living + stillborn + abortions exceeds Parity, or gestation month exceeds 9</t>
+          <t>block enrolment when Parity exceeds Gravida, the subject is male, or the subject is under a minimum age (e.g. 16)</t>
         </is>
       </c>
     </row>
@@ -24129,7 +24129,7 @@
       </c>
       <c r="D12" s="13" t="inlineStr">
         <is>
-          <t>when followup is marked done, require at least one of the audio or text fields to be filled; otherwise require a reason</t>
+          <t>block saving when a reason field is empty, and additionally require evidence fields when a yes/no field marks the activity done</t>
         </is>
       </c>
     </row>
@@ -24193,7 +24193,7 @@
       </c>
       <c r="D14" s="13" t="inlineStr">
         <is>
-          <t>use RuleCondition to express validation declaratively - push errors when conditions on age, gender, or registration values are not met</t>
+          <t>block saving when none of a required set of registration values is provided (e.g. at least one of Father/Mother/Guardian name)</t>
         </is>
       </c>
     </row>
@@ -24359,7 +24359,7 @@
       </c>
       <c r="D18" s="13" t="inlineStr">
         <is>
-          <t>block enrolment for individuals registered before a cutoff year</t>
+          <t>block enrolment when the subject was registered in or before a cutoff year and the enrolment is being recorded after that year (e.g. 2020)</t>
         </is>
       </c>
     </row>
@@ -24400,44 +24400,15 @@
     <row r="20">
       <c r="A20" s="13" t="inlineStr">
         <is>
-          <t>Atul Foundation</t>
+          <t>Goonj</t>
         </is>
       </c>
       <c r="B20" s="13" t="inlineStr">
         <is>
-          <t>Individual Registration</t>
+          <t>Village Registration</t>
         </is>
       </c>
       <c r="C20" s="13" t="inlineStr">
-        <is>
-          <t>"use strict";
- ({params, imports}) =&gt; {
-  const individual = params.entity;
-  const validationResults = [];
-  //use imports.common.createValidationError('sample error') to create validation error and push it to validationResults
-  console.log('individual---&gt;',individual);
-  return validationResults;
- };</t>
-        </is>
-      </c>
-      <c r="D20" s="13" t="inlineStr">
-        <is>
-          <t>validation passes for all entries (placeholder - returns no errors)</t>
-        </is>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" s="13" t="inlineStr">
-        <is>
-          <t>Goonj</t>
-        </is>
-      </c>
-      <c r="B21" s="13" t="inlineStr">
-        <is>
-          <t>Village Registration</t>
-        </is>
-      </c>
-      <c r="C21" s="13" t="inlineStr">
         <is>
           <t>"use strict";
  ({params, imports}) =&gt; {
@@ -24489,62 +24460,24 @@
  };</t>
         </is>
       </c>
-      <c r="D21" s="13" t="inlineStr">
+      <c r="D20" s="13" t="inlineStr">
         <is>
           <t>block creating a duplicate village registration for the same location</t>
         </is>
       </c>
     </row>
-    <row r="22">
-      <c r="A22" s="13" t="inlineStr">
-        <is>
-          <t>Gram Seva Trust</t>
-        </is>
-      </c>
-      <c r="B22" s="13" t="inlineStr">
-        <is>
-          <t>Diabetes/HTN Followup Encounter</t>
-        </is>
-      </c>
-      <c r="C22" s="13" t="inlineStr">
-        <is>
-          <t>"use strict";
- ({params, imports}) =&gt; {
-  const programEncounter = params.entity;
-  const moment = imports.moment;
-  const validationResults = [];
-  let oldSelectedDate = programEncounter.getObservationReadableValue("717128d8-fa2b-4943-95aa-e3d1f3ef2cd1");
-  if (oldSelectedDate) {
-  oldSelectedDate = moment(oldSelectedDate, "YYYY-MM-DD", true).format("YYYY-MM-DD");
-  }
-  let selectedDate = programEncounter.getObservationReadableValue("fbf6eee4-ed36-4570-a305-e97eacd50136");
-  if (selectedDate) {
-  selectedDate = moment(selectedDate, "YYYY-MM-DD", true).format("YYYY-MM-DD");
-  }
-  console.log('oldSelectedDate---&gt;',oldSelectedDate);
-  console.log('selectedDate----&gt;',selectedDate);
-  return validationResults;
- };</t>
-        </is>
-      </c>
-      <c r="D22" s="13" t="inlineStr">
-        <is>
-          <t>block saving when an observation value differs from the previously recorded value</t>
-        </is>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" s="13" t="inlineStr">
+    <row r="21">
+      <c r="A21" s="13" t="inlineStr">
         <is>
           <t>Durga India</t>
         </is>
       </c>
-      <c r="B23" s="13" t="inlineStr">
+      <c r="B21" s="13" t="inlineStr">
         <is>
           <t>Session Encounter</t>
         </is>
       </c>
-      <c r="C23" s="13" t="inlineStr">
+      <c r="C21" s="13" t="inlineStr">
         <is>
           <t>"use strict";
  ({params, imports}) =&gt; {
@@ -24564,24 +24497,24 @@
  };</t>
         </is>
       </c>
-      <c r="D23" s="13" t="inlineStr">
-        <is>
-          <t>block saving when the encounter is still awaiting approval</t>
-        </is>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" s="13" t="inlineStr">
+      <c r="D21" s="13" t="inlineStr">
+        <is>
+          <t>block saving an encounter when its date is after a previously-completed terminal/endline encounter for the same subject (e.g. block a session visit dated after the cohort endline)</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="13" t="inlineStr">
         <is>
           <t>CES</t>
         </is>
       </c>
-      <c r="B24" s="13" t="inlineStr">
+      <c r="B22" s="13" t="inlineStr">
         <is>
           <t>Tuberculosis Exit</t>
         </is>
       </c>
-      <c r="C24" s="13" t="inlineStr">
+      <c r="C22" s="13" t="inlineStr">
         <is>
           <t>"use strict";
  ({params, imports}) =&gt; {
@@ -24599,24 +24532,24 @@
  };</t>
         </is>
       </c>
-      <c r="D24" s="13" t="inlineStr">
-        <is>
-          <t>require a date of death observation when the program is being exited</t>
-        </is>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" s="13" t="inlineStr">
+      <c r="D22" s="13" t="inlineStr">
+        <is>
+          <t>block exiting the program when the recorded date of death is before the enrolment date</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="13" t="inlineStr">
         <is>
           <t>CES</t>
         </is>
       </c>
-      <c r="B25" s="13" t="inlineStr">
+      <c r="B23" s="13" t="inlineStr">
         <is>
           <t>Periodic check-in</t>
         </is>
       </c>
-      <c r="C25" s="13" t="inlineStr">
+      <c r="C23" s="13" t="inlineStr">
         <is>
           <t>"use strict";
  ({params, imports}) =&gt; {
@@ -24636,7 +24569,7 @@
  };</t>
         </is>
       </c>
-      <c r="D25" s="13" t="inlineStr">
+      <c r="D23" s="13" t="inlineStr">
         <is>
           <t>block saving when the visit date is earlier than the treatment-start date for this enrolment</t>
         </is>
@@ -25647,7 +25580,7 @@
     <outlinePr summaryBelow="0" summaryRight="0"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D9"/>
+  <dimension ref="A1:D8"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="12.63" defaultRowHeight="15" customHeight="1"/>
   <cols>
     <col width="22" customWidth="1" style="11" min="1" max="1"/>
@@ -25756,49 +25689,22 @@
       </c>
       <c r="D3" s="13" t="inlineStr">
         <is>
-          <t>allow editing the cancellation only within the same month as the cancel date</t>
+          <t>block editing a cancelled encounter once its scheduled month has passed</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="13" t="inlineStr">
         <is>
-          <t>IPH Sickle Cell</t>
+          <t>Goonj</t>
         </is>
       </c>
       <c r="B4" s="13" t="inlineStr">
         <is>
-          <t>Participant Initial Registration Form</t>
+          <t>Quarterly Planning</t>
         </is>
       </c>
       <c r="C4" s="13" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  "use strict";
- ({params, imports}) =&gt; {
-  const {entity, form, services, entityContext, myUserGroups, userInfo} = params;
-  const output = {}; // https://avni.readme.io/docs/writing-rules#16-edit-form-rule
-  return output;
- };</t>
-        </is>
-      </c>
-      <c r="D4" s="13" t="inlineStr">
-        <is>
-          <t>always allow editing (placeholder rule)</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="13" t="inlineStr">
-        <is>
-          <t>Goonj</t>
-        </is>
-      </c>
-      <c r="B5" s="13" t="inlineStr">
-        <is>
-          <t>Quarterly Planning</t>
-        </is>
-      </c>
-      <c r="C5" s="13" t="inlineStr">
         <is>
           <t>"use strict";
  ({params, imports}) =&gt; {
@@ -25816,24 +25722,24 @@
  };</t>
         </is>
       </c>
-      <c r="D5" s="13" t="inlineStr">
+      <c r="D4" s="13" t="inlineStr">
         <is>
           <t>block editing once the form is marked as Reviewed</t>
         </is>
       </c>
     </row>
-    <row r="6">
-      <c r="A6" s="13" t="inlineStr">
+    <row r="5">
+      <c r="A5" s="13" t="inlineStr">
         <is>
           <t>JSSCP</t>
         </is>
       </c>
-      <c r="B6" s="13" t="inlineStr">
+      <c r="B5" s="13" t="inlineStr">
         <is>
           <t>Referral Communication Encounter</t>
         </is>
       </c>
-      <c r="C6" s="13" t="inlineStr">
+      <c r="C5" s="13" t="inlineStr">
         <is>
           <t xml:space="preserve"> "use strict";
  ({params, imports}) =&gt; {
@@ -25860,24 +25766,24 @@
  };</t>
         </is>
       </c>
-      <c r="D6" s="13" t="inlineStr">
-        <is>
-          <t>allow editing only by users whose user-group matches the UUID recorded on the encounter</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="13" t="inlineStr">
+      <c r="D5" s="13" t="inlineStr">
+        <is>
+          <t>allow editing only by users whose group matches the group recorded on the encounter</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="13" t="inlineStr">
         <is>
           <t>Maitrayana</t>
         </is>
       </c>
-      <c r="B7" s="13" t="inlineStr">
+      <c r="B6" s="13" t="inlineStr">
         <is>
           <t>YPI Pragati Lifeskill Session Attendance Encounter</t>
         </is>
       </c>
-      <c r="C7" s="13" t="inlineStr">
+      <c r="C6" s="13" t="inlineStr">
         <is>
           <t xml:space="preserve">  "use strict";
  ({params, imports}) =&gt; {
@@ -25895,24 +25801,24 @@
  };</t>
         </is>
       </c>
-      <c r="D7" s="13" t="inlineStr">
+      <c r="D6" s="13" t="inlineStr">
         <is>
           <t>allow editing only by the assigned role within N days of the encounter date</t>
         </is>
       </c>
     </row>
-    <row r="8">
-      <c r="A8" s="13" t="inlineStr">
+    <row r="7">
+      <c r="A7" s="13" t="inlineStr">
         <is>
           <t>Goonj</t>
         </is>
       </c>
-      <c r="B8" s="13" t="inlineStr">
+      <c r="B7" s="13" t="inlineStr">
         <is>
           <t>Village Registration</t>
         </is>
       </c>
-      <c r="C8" s="13" t="inlineStr">
+      <c r="C7" s="13" t="inlineStr">
         <is>
           <t xml:space="preserve"> "use strict";
  ({params, imports}) =&gt; {
@@ -25934,24 +25840,24 @@
  };</t>
         </is>
       </c>
-      <c r="D8" s="13" t="inlineStr">
-        <is>
-          <t>allow editing only by the original creator within N days, reloading from DB to confirm the latest creator</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="13" t="inlineStr">
+      <c r="D7" s="13" t="inlineStr">
+        <is>
+          <t>allow editing only by the original creator within N days of the registration</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="13" t="inlineStr">
         <is>
           <t>Durga India</t>
         </is>
       </c>
-      <c r="B9" s="13" t="inlineStr">
+      <c r="B8" s="13" t="inlineStr">
         <is>
           <t>Participant Registration</t>
         </is>
       </c>
-      <c r="C9" s="13" t="inlineStr">
+      <c r="C8" s="13" t="inlineStr">
         <is>
           <t xml:space="preserve"> "use strict";
  ({params, imports}) =&gt; {
@@ -26019,9 +25925,9 @@
  };</t>
         </is>
       </c>
-      <c r="D9" s="13" t="inlineStr">
-        <is>
-          <t>allow editing only when the encounter is in 'Submission for approval' state and the user has the matching role</t>
+      <c r="D8" s="13" t="inlineStr">
+        <is>
+          <t>allow editing based on the cohort's approval workflow state (admins always; approved blocks non-admins; pending allows only the approver role; rejected re-opens editing), and restrict lower roles to records they created</t>
         </is>
       </c>
     </row>
@@ -44047,7 +43953,7 @@
     <outlinePr summaryBelow="0" summaryRight="0"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D15"/>
+  <dimension ref="A1:D13"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="12.63" defaultRowHeight="15" customHeight="1"/>
   <cols>
     <col width="22" customWidth="1" style="11" min="1" max="1"/>
@@ -44112,7 +44018,7 @@
       </c>
       <c r="D2" s="13" t="inlineStr">
         <is>
-          <t>use the complicationsBuilder DSL to add a clinical complication when specified answers are selected on the form</t>
+          <t>show which clinical complications apply based on the answers selected on the form</t>
         </is>
       </c>
     </row>
@@ -44218,7 +44124,7 @@
       </c>
       <c r="D3" s="13" t="inlineStr">
         <is>
-          <t>compute WFA, HFA, and WFH z-scores from height, weight, age, and sex, then classify each as normal / MAM / SAM</t>
+          <t>classify the subject's nutritional status (WFA/HFA/WFH) from height, weight, age, sex, and flag growth faltering when weight gain since the prior visit is low</t>
         </is>
       </c>
     </row>
@@ -44271,7 +44177,7 @@
       </c>
       <c r="D4" s="13" t="inlineStr">
         <is>
-          <t>compute BMI from height and weight and bucket into underweight / normal / overweight / obese</t>
+          <t>show the subject's BMI category (underweight / normal / overweight / obese) based on recorded height and weight</t>
         </is>
       </c>
     </row>
@@ -44395,7 +44301,7 @@
       </c>
       <c r="D5" s="13" t="inlineStr">
         <is>
-          <t>carry forward the most recent observation value from the previous completed visit into this encounter's decisions</t>
+          <t>classify multiple clinical risks (anaemia, malnutrition, sickle cell, school dropout, mental-health flag) from recorded observation values, and propagate selected values to enrolment when the visit is the latest</t>
         </is>
       </c>
     </row>
@@ -44466,7 +44372,7 @@
       </c>
       <c r="D6" s="13" t="inlineStr">
         <is>
-          <t>set a follow-up flag based on whether a clinical condition (sickle cell, epilepsy, diabetes) was observed in this visit</t>
+          <t>record the subject's current medication regimen (medicines and dosage details) as decisions, carrying values forward from prior visits when the regimen continues unchanged</t>
         </is>
       </c>
     </row>
@@ -44498,7 +44404,7 @@
       </c>
       <c r="D7" s="13" t="inlineStr">
         <is>
-          <t>when a date of death is recorded, set the individual's status to Dead and write the death date back to registration</t>
+          <t>set the subject's life status to Dead and propagate the date of death to registration when a date of death is recorded on exit</t>
         </is>
       </c>
     </row>
@@ -44526,7 +44432,7 @@
       </c>
       <c r="D8" s="13" t="inlineStr">
         <is>
-          <t>set the individual's status to Alive on registration</t>
+          <t>set the subject's initial life status (Alive) on registration</t>
         </is>
       </c>
     </row>
@@ -44557,7 +44463,7 @@
       </c>
       <c r="D9" s="13" t="inlineStr">
         <is>
-          <t>copy selected observations from this form into the registration / encounter decisions verbatim</t>
+          <t>surface selected form observations as decisions without transformation</t>
         </is>
       </c>
     </row>
@@ -44590,7 +44496,7 @@
       </c>
       <c r="D10" s="13" t="inlineStr">
         <is>
-          <t>copy observations to decisions only when a gating answer (e.g. consent == Yes) is selected</t>
+          <t>surface selected observations as decisions only when a gating answer (e.g. consent == Yes) is recorded</t>
         </is>
       </c>
     </row>
@@ -44628,7 +44534,7 @@
       </c>
       <c r="D11" s="13" t="inlineStr">
         <is>
-          <t>record the username, full name, and UUID of the user who entered the encounter into registration decisions</t>
+          <t>record the user who entered the registration as an audit decision</t>
         </is>
       </c>
     </row>
@@ -44674,7 +44580,7 @@
       </c>
       <c r="D12" s="13" t="inlineStr">
         <is>
-          <t>record who entered the encounter, when it was entered, and lock the entry date across subsequent edits</t>
+          <t>record creator name and username on every save, and stamp the registration date only on the first save</t>
         </is>
       </c>
     </row>
@@ -44759,251 +44665,7 @@
       </c>
       <c r="D13" s="13" t="inlineStr">
         <is>
-          <t>classify the subject (e.g. risk level, eligibility band) using RuleCondition match logic and push the result to decisions</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="13" t="inlineStr">
-        <is>
-          <t>JNPCT</t>
-        </is>
-      </c>
-      <c r="B14" s="13" t="inlineStr">
-        <is>
-          <t>Child PNC Cluster Incahrge</t>
-        </is>
-      </c>
-      <c r="C14" s="13" t="inlineStr">
-        <is>
-          <t>"use strict";
- ({params, imports}) =&gt; {
-  const programEncounter = params.entity;
-  const decisions = params.decisions;
-  const age = programEncounter.programEnrolment.individual.getAgeInMonths();
-  const decisionBuilder = new imports.rulesConfig.complicationsBuilder({
-  programEncounter: programEncounter,
-  complicationsConcept: "Counsel mother"
-  });
-  decisionBuilder.addComplication("Keep child warm in cloths")
-  .when.valueInEncounter("Is there active movement of hands and legs?")
-  .is.no;
-  decisionBuilder.addComplication("Keep child warm in cloths")
-  .when.valueInEncounter("Is there any life threatening abnormality?")
-  .is.no;
-  decisionBuilder.addComplication("Keep child in 3-4 folded cloths")
-  .when.valueInEncounter("Is infant coverred with 3-4 folded cloth?")
-  .containsAnswerConceptNameOtherThan("Properly covered and head also covered");
-  decisionBuilder.addComplication("Give PCM")
-  .when.valueInEncounter("Temperature of infant")
-  .is.greaterThan(37.5);
-  decisionBuilder.addComplication("Keep child warm in cloths")
-  .when.valueInEncounter("Temperature of infant")
-  .is.lessThanOrEqualTo(35.5);
-  decisionBuilder.addComplication("Give PCM")
-  .when.valueInEncounter("How you feel infants temprature on touch?")
-  .containsAnswerConceptName("Abdomen and limbs all feel hot on touch");
-  decisionBuilder.addComplication("Keep child warm in cloths")
-  .when.valueInEncounter("How you feel infants temprature on touch?")
-  .containsAnswerConceptName("Abdomen and limbs feel cold on touch");
-  decisionBuilder.addComplication("apply 0.25%GV lotion, give first dose of cotri")
-  .when.valueInEncounter("Condition of umbelicus")
-  .containsAnswerConceptNameOtherThan("Normal");
-  decisionBuilder.addComplication("Expain mother for exclusive breastfeeding")
-  .when.valueInEncounter("Is there anything given other than breastfeeding for infant")
-  .is.yes;
-  decisionBuilder.addComplication("Expain mother for breastfeeding more than 10 times")
-  .when.valueInEncounter("How many times breastfeeding given to child in last 24 hours")
-  .is.lessThan(8);
-  decisionBuilder.addComplication("Expain mother to increase frequency of breastfeeding")
-  .when.valueInEncounter("In last 24 hours, for how many times infant passes urine?")
-  .containsAnswerConceptName("Less than 5 times");
-  decisionBuilder.addComplication("Give primary treatment")
-  .when.valueInEncounter("Is there bleeding from any part of infant's body?")
-  .is.yes;
-  decisionBuilder.addComplication("Give primary treatment")
-  .when.valueInEncounter("Is infant vomiting?")
-  .is.yes;
-  decisionBuilder.addComplication("Give primary treatment")
-  .when.valueInEncounter("Does infant's abdomen look gasious?")
-  .is.yes;
-  decisionBuilder.addComplication("Give primary treatment")
-  .when.valueInEncounter("Does infant looks icteric?")
-  .is.yes;
-  decisionBuilder.addComplication("Give primary treatment")
-  .when.valueInEncounter("Does infant looks cynosed?")
-  .is.yes;
-  decisionBuilder.addComplication("Give primary treatment")
-  .when.valueInEncounter("Does infant looks abnormal?")
-  .is.yes;
-  decisionBuilder.addComplication("Give primary treatment")
-  .when.valueInEncounter("Is the infant's mouth cleft pallet seen?")
-  .is.yes;
-  decisionBuilder.addComplication("Give primary treatment")
-  .when.valueInEncounter("Is there visible tumor on back or on head of infant?")
-  .is.yes;
-  decisionBuilder.addComplication("Give primary treatment")
-  .when.valueInEncounter("Is foam coming from infant's mouth continuously?")
-  .is.yes;
-  decisionBuilder.addComplication("Give primary treatment")
-  .when.valueInEncounter("Does infant has watery diarrhoea?")
-  .is.yes;
-  decisionBuilder.addComplication("Apply 0.25 % GV lotion two times a day")
-  .when.valueInEncounter("Is oral ulcer or thrush seen in infant's mouth")
-  .is.yes;
-  decisionBuilder
-  .addComplication("If 10 or above pustules are present then give primary treatment and refer")
-  .when.valueInEncounter("If yes, then how many visible pustules are on the body")
-  .containsAnswerConceptName("10 or more than 10");
-  decisionBuilder
-  .addComplication("If less than 10 pustule then apply 0.5% GV lotion and give cotri syrup two times for 5 days").when.valueInEncounter("If yes, then how many visible pustules are on the body")
-  .containsAnswerConceptName("Less than 10");
-  decisions.encounterDecisions.push(decisionBuilder.getComplications());
-  const complicationsBuilder = new imports.rulesConfig.complicationsBuilder({
-  programEncounter: programEncounter,
-  complicationsConcept: "Refer to the hospital for"
-  });
-  complicationsBuilder.addComplication("Not breathing properly")
-  .when.valueInEncounter("Whether child breathing regularly?")
-  .is.no;
-  complicationsBuilder.addComplication("No Active Movement of hands and legs")
-  .when.valueInEncounter("Is there active movement of hands and legs?")
-  .is.no;
-  complicationsBuilder.addComplication("Not paases stool and urine within 24 hour")
-  .when.valueInEncounter("Does child paases stool and urine within 24 hour")
-  .is.no;
-  complicationsBuilder.addComplication("Life threatening abnormality")
-  .when.valueInEncounter("Is there any life threatening abnormality?")
-  .is.yes;
-  complicationsBuilder.addComplication("palate/lips in child's mouth")
-  .when.valueInEncounter("Examine for cleft palate/lips in child's mouth?")
-  .is.yes;
-  complicationsBuilder.addComplication("Blood coming out from part of body")
-  .when.valueInEncounter("Is blood coming out from any part of body?")
-  .is.yes;
-  complicationsBuilder.addComplication("There is visible jaundice")
-  .when.valueInEncounter("Is there visible jaundice?")
-  .is.yes;
-  complicationsBuilder.addComplication("High respiratory rate")
-  .when.valueInEncounter("Child Respiratory Rate")
-  .is.greaterThan(50).and.whenItem(age &lt; 13).is.truthy
-  .and.whenItem(age &gt; 2).is.truthy;
-  complicationsBuilder.addComplication("High respiratory rate")
-  .when.valueInEncounter("Child Respiratory Rate")
-  .is.greaterThan(40).and.whenItem(age &gt; 12).is.truthy;
-  complicationsBuilder.addComplication("High respiratory rate")
-  .when.valueInEncounter("Child Respiratory Rate")
-  .is.greaterThan(60).and.whenItem(age &lt; 2).is.truthy;
-  complicationsBuilder.addComplication("There is grunting sound")
-  .when.valueInEncounter("Is there any grunting sound?")
-  .is.yes;
-  complicationsBuilder.addComplication("Abnormal Color")
-  .when.valueInEncounter("How is the colour of infant")
-  .containsAnswerConceptNameOtherThan("Pinkish");
-  complicationsBuilder.addComplication("Less Infants Movement")
-  .when.valueInEncounter("Look at the infants movement")
-  .containsAnswerConceptNameOtherThan("Normal");
-  complicationsBuilder.addComplication("High Fever")
-  .when.valueInEncounter("Temperature of infant")
-  .is.greaterThan(37.5);
-  complicationsBuilder.addComplication("Low Temperature of infant")
-  .when.valueInEncounter("Temperature of infant")
-  .is.lessThanOrEqualTo(35.5);
-  complicationsBuilder.addComplication("High Temperature of infant")
-  .when.valueInEncounter("How you feel infants temprature on touch?")
-  .containsAnswerConceptName("Abdomen and limbs all feel hot on touch");
-  complicationsBuilder.addComplication("Low Temperature of infant")
-  .when.valueInEncounter("How you feel infants temprature on touch?")
-  .containsAnswerConceptName("Abdomen and limbs feel cold on touch");
-  complicationsBuilder.addComplication("Abnormal Condition of umbelicus")
-  .when.valueInEncounter("Condition of umbelicus")
-  .containsAnswerConceptNameOtherThan("Normal");
-  complicationsBuilder.addComplication("Abnormal attachment while sucking")
-  .when.valueInEncounter("How is the infant attachment while sucking?")
-  .containsAnswerConceptNameOtherThan("Good - Normal");
-  complicationsBuilder.addComplication("Difficulty in breastfeeding")
-  .when.valueInEncounter("Does infant has any difficulty in breastfeeding?")
-  .is.yes;
-  complicationsBuilder.addComplication("Bleeding from part of body")
-  .when.valueInEncounter("Is there bleeding from any part of infant's body?")
-  .is.yes;
-  complicationsBuilder.addComplication("Infant vomiting")
-  .when.valueInEncounter("Is infant vomiting?")
-  .is.yes;
-  complicationsBuilder.addComplication("infant's abdomen look gasious")
-  .when.valueInEncounter("Does infant's abdomen look gasious?")
-  .is.yes;
-  complicationsBuilder.addComplication("infant looks icteric")
-  .when.valueInEncounter("Does infant looks icteric?")
-  .is.yes;
-  complicationsBuilder.addComplication("infant looks cynosed")
-  .when.valueInEncounter("Does infant looks cynosed?")
-  .is.yes;
-  complicationsBuilder.addComplication("infant looks abnormal")
-  .when.valueInEncounter("Does infant looks abnormal?")
-  .is.yes;
-  complicationsBuilder.addComplication("cleft pallet seen in infant's mouth")
-  .when.valueInEncounter("Is the infant's mouth cleft pallet seen?")
-  .is.yes;
-  complicationsBuilder.addComplication("there is visible tumor")
-  .when.valueInEncounter("Is there visible tumor on back or on head of infant?")
-  .is.yes;
-  complicationsBuilder.addComplication("Continuously foam is coming from mouth")
-  .when.valueInEncounter("Is foam coming from infant's mouth continuously?")
-  .is.yes;
-  complicationsBuilder.addComplication("infant has watery diarrhoea")
-  .when.valueInEncounter("Does infant has watery diarrhoea?")
-  .is.yes;
-  const medicinedecisionBuilder = new imports.rulesConfig.complicationsBuilder({
-  programEncounter: programEncounter,
-  complicationsConcept: "medicine recommendations"
-  });
-  medicinedecisionBuilder
-  .addComplication("If less than 10 pustule then give Cotrimoxazole with 1.5 ml of dosage")
-  .when.valueInEncounter("If yes, then how many visible pustules are on the body")
-  .containsAnswerConceptName("Less than 10").and.whenItem(age &lt; 1).is.truthy;
-  medicinedecisionBuilder
-  .addComplication("If less than 10 pustule then give Cotrimoxazole with 2.5 ml of dosage")
-  .when.valueInEncounter("If yes, then how many visible pustules are on the body")
-  .containsAnswerConceptName("Less than 10").and.whenItem(age &lt; 2).is.truthy
-  .and.whenItem(age &gt;= 1).is.truthy;
-  decisions.encounterDecisions.push(complicationsBuilder.getComplications());
-  decisions.encounterDecisions.push(medicinedecisionBuilder.getComplications());
-  return decisions;
- };</t>
-        </is>
-      </c>
-      <c r="D14" s="13" t="inlineStr">
-        <is>
-          <t>bucket the subject into an age category using getAgeInYears / getAgeInMonths and push the bucket to decisions</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="13" t="inlineStr">
-        <is>
-          <t>SNCU</t>
-        </is>
-      </c>
-      <c r="B15" s="13" t="inlineStr">
-        <is>
-          <t>Child Enrolment</t>
-        </is>
-      </c>
-      <c r="C15" s="13" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  "use strict";
- ({params, imports}) =&gt; {
-  const programEnrolment = params.entity;
-  const decisions = params.decisions;
-  //create complicationBuilder using programEnrolment and then push to enrolmentDecisions array.
-  return decisions;
- };</t>
-        </is>
-      </c>
-      <c r="D15" s="13" t="inlineStr">
-        <is>
-          <t>decisions pass through unchanged (placeholder rule)</t>
+          <t>backfill identity-card numbers (e.g. Aadhaar, Ration Card, CMCHIS) onto the registration from an upstream encounter when the registration field is empty</t>
         </is>
       </c>
     </row>

</xml_diff>